<commit_message>
Update House model inputs and outputs
</commit_message>
<xml_diff>
--- a/inputs/House Model Data.xlsx
+++ b/inputs/House Model Data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/benyelin/Desktop/Desktop - Ben’s MacBook Air/house_model_python/inputs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF9F29D5-7359-3640-BA9E-CB071328F0CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAB5DC30-0C5D-914F-936B-C4393B01B63A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1460" yWindow="1560" windowWidth="27640" windowHeight="16940" xr2:uid="{9CA4CF23-00BE-4A4E-B0A3-B27FE202FE9A}"/>
   </bookViews>
@@ -73,7 +73,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5234" uniqueCount="813">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5362" uniqueCount="898">
   <si>
     <t>State</t>
   </si>
@@ -2512,6 +2512,261 @@
   </si>
   <si>
     <t>Bartie, Thurmond</t>
+  </si>
+  <si>
+    <t>Nez, Jonathan</t>
+  </si>
+  <si>
+    <t>Jasser, Zuhdi</t>
+  </si>
+  <si>
+    <t>Mendoza, JoAnn</t>
+  </si>
+  <si>
+    <t>Butierez, Daniel</t>
+  </si>
+  <si>
+    <t>Hamadeh, Abraham</t>
+  </si>
+  <si>
+    <t>Sterbinsky, Danielle</t>
+  </si>
+  <si>
+    <t>Jones, Eric</t>
+  </si>
+  <si>
+    <t>Frese, Jeffrey</t>
+  </si>
+  <si>
+    <t>Hernandez, Melissa</t>
+  </si>
+  <si>
+    <t>Soule, Peter</t>
+  </si>
+  <si>
+    <t>Morales, Christian</t>
+  </si>
+  <si>
+    <t>Hollowell, Amanda</t>
+  </si>
+  <si>
+    <t>Kingston, James</t>
+  </si>
+  <si>
+    <t>Martin, Kevin</t>
+  </si>
+  <si>
+    <t>Kozycki, Tony</t>
+  </si>
+  <si>
+    <t>DeLancy, Pamela</t>
+  </si>
+  <si>
+    <t>Cowan, John</t>
+  </si>
+  <si>
+    <t>Smith, Ceretta</t>
+  </si>
+  <si>
+    <t>Dunlap, Matthew</t>
+  </si>
+  <si>
+    <t>Pino, Rosemary</t>
+  </si>
+  <si>
+    <t>Gallant, Christopher</t>
+  </si>
+  <si>
+    <t>Halpin, Patrick</t>
+  </si>
+  <si>
+    <t>LePetri, Michael</t>
+  </si>
+  <si>
+    <t>Driscoll, Jeanine</t>
+  </si>
+  <si>
+    <t>Marsh, George</t>
+  </si>
+  <si>
+    <t>Chou, Joseph</t>
+  </si>
+  <si>
+    <t>Valdez, Claire</t>
+  </si>
+  <si>
+    <t>Rivera, Mevlin</t>
+  </si>
+  <si>
+    <t>Mizrahi, Lewis</t>
+  </si>
+  <si>
+    <t>Anabilah-Azuman, Joel</t>
+  </si>
+  <si>
+    <t>Lander, Brad</t>
+  </si>
+  <si>
+    <t>Moore, Jennifer</t>
+  </si>
+  <si>
+    <t>DeCillis, Michael</t>
+  </si>
+  <si>
+    <t>Lasher, Micah</t>
+  </si>
+  <si>
+    <t>Shinkle, Caroline</t>
+  </si>
+  <si>
+    <t>Chavalier, Daraliza Avila</t>
+  </si>
+  <si>
+    <t>Williams, Manual</t>
+  </si>
+  <si>
+    <t>Hysanaj, Diamant</t>
+  </si>
+  <si>
+    <t>Sapaskis, Stylo</t>
+  </si>
+  <si>
+    <t>Cinquemani, Joseph</t>
+  </si>
+  <si>
+    <t>Conley, Cait</t>
+  </si>
+  <si>
+    <t>Auringer, Jackie</t>
+  </si>
+  <si>
+    <t>Oberacker, Peter</t>
+  </si>
+  <si>
+    <t>Ambrosio, Ralph</t>
+  </si>
+  <si>
+    <t>Gendebien, Blake</t>
+  </si>
+  <si>
+    <t>Constantino, Anthony</t>
+  </si>
+  <si>
+    <t>Buller, Kailee</t>
+  </si>
+  <si>
+    <t>Gies, Aaron</t>
+  </si>
+  <si>
+    <t>Ellman, Alissa</t>
+  </si>
+  <si>
+    <t>Morelle, Joseph</t>
+  </si>
+  <si>
+    <t>McIntyre, Virginia</t>
+  </si>
+  <si>
+    <t>Hannon, Dennis</t>
+  </si>
+  <si>
+    <t>Scwhartz, Dan</t>
+  </si>
+  <si>
+    <t>Boafo, Adrian</t>
+  </si>
+  <si>
+    <t>Wallace, Dave</t>
+  </si>
+  <si>
+    <t>Flowers, Bernard</t>
+  </si>
+  <si>
+    <t>McDermott, George</t>
+  </si>
+  <si>
+    <t>Chaffee, Chris</t>
+  </si>
+  <si>
+    <t>Ficker, Robin</t>
+  </si>
+  <si>
+    <t>Collier, Scott</t>
+  </si>
+  <si>
+    <t>Riley, Cheryl</t>
+  </si>
+  <si>
+    <t>Lacore, Nancy</t>
+  </si>
+  <si>
+    <t>Honeycutt, Jenny</t>
+  </si>
+  <si>
+    <t>Khalifa, Zyon</t>
+  </si>
+  <si>
+    <t>McAdams, Ben</t>
+  </si>
+  <si>
+    <t>Owen, Riley</t>
+  </si>
+  <si>
+    <t>Crosby, Peter</t>
+  </si>
+  <si>
+    <t>Udell, Kent</t>
+  </si>
+  <si>
+    <t>Larsen, Jonny</t>
+  </si>
+  <si>
+    <t>Feely, Jay</t>
+  </si>
+  <si>
+    <t>Lamb, Mike</t>
+  </si>
+  <si>
+    <t>Lee, Elizabeth</t>
+  </si>
+  <si>
+    <t>Greene-Placentia, Bernadette</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Glenn, Nicholas </t>
+  </si>
+  <si>
+    <t>Kiros, Melat</t>
+  </si>
+  <si>
+    <t>Peterson, Christy</t>
+  </si>
+  <si>
+    <t>Dennison, Kelley</t>
+  </si>
+  <si>
+    <t>Romero, Dwayne</t>
+  </si>
+  <si>
+    <t>Laubaucher, Eileen</t>
+  </si>
+  <si>
+    <t>Killin, Jessica</t>
+  </si>
+  <si>
+    <t>Tewahade, Mel</t>
+  </si>
+  <si>
+    <t>Bennett, Timothy</t>
+  </si>
+  <si>
+    <t>Rutinel, Manny</t>
+  </si>
+  <si>
+    <t>Shah, Amish</t>
+  </si>
+  <si>
+    <t>Hammer, Trygve</t>
   </si>
 </sst>
 </file>
@@ -2945,7 +3200,7 @@
     <col min="3" max="4" width="29.83203125" customWidth="1"/>
     <col min="5" max="6" width="20.6640625" style="3" customWidth="1"/>
     <col min="7" max="7" width="30.1640625" style="3" customWidth="1"/>
-    <col min="8" max="8" width="23.33203125" customWidth="1"/>
+    <col min="8" max="8" width="36.5" customWidth="1"/>
     <col min="9" max="10" width="24.1640625" customWidth="1"/>
     <col min="11" max="11" width="13.6640625" hidden="1" customWidth="1"/>
     <col min="12" max="12" width="18.6640625" hidden="1" customWidth="1"/>
@@ -3380,6 +3635,12 @@
         <f t="shared" si="0"/>
         <v>5.3000000000000007</v>
       </c>
+      <c r="H10" s="4" t="s">
+        <v>896</v>
+      </c>
+      <c r="I10" s="4" t="s">
+        <v>882</v>
+      </c>
       <c r="K10" t="s">
         <v>675</v>
       </c>
@@ -3402,7 +3663,7 @@
         <v>700</v>
       </c>
       <c r="T10" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="11" spans="1:22" x14ac:dyDescent="0.2">
@@ -3429,6 +3690,12 @@
         <f t="shared" si="0"/>
         <v>-6.5</v>
       </c>
+      <c r="H11" s="4" t="s">
+        <v>813</v>
+      </c>
+      <c r="I11" t="s">
+        <v>20</v>
+      </c>
       <c r="K11" t="s">
         <v>675</v>
       </c>
@@ -3451,7 +3718,7 @@
         <v>700</v>
       </c>
       <c r="T11" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="12" spans="1:22" x14ac:dyDescent="0.2">
@@ -3478,6 +3745,12 @@
         <f t="shared" si="0"/>
         <v>48</v>
       </c>
+      <c r="H12" t="s">
+        <v>21</v>
+      </c>
+      <c r="I12" s="4" t="s">
+        <v>886</v>
+      </c>
       <c r="K12" t="s">
         <v>675</v>
       </c>
@@ -3500,7 +3773,7 @@
         <v>700</v>
       </c>
       <c r="T12" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="13" spans="1:22" x14ac:dyDescent="0.2">
@@ -3527,6 +3800,12 @@
         <f t="shared" si="0"/>
         <v>15.7</v>
       </c>
+      <c r="H13" t="s">
+        <v>22</v>
+      </c>
+      <c r="I13" s="4" t="s">
+        <v>814</v>
+      </c>
       <c r="K13" t="s">
         <v>675</v>
       </c>
@@ -3549,7 +3828,7 @@
         <v>700</v>
       </c>
       <c r="T13" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="14" spans="1:22" x14ac:dyDescent="0.2">
@@ -3576,6 +3855,12 @@
         <f t="shared" si="0"/>
         <v>-11.499999999999998</v>
       </c>
+      <c r="H14" s="4" t="s">
+        <v>884</v>
+      </c>
+      <c r="I14" s="4" t="s">
+        <v>883</v>
+      </c>
       <c r="K14" t="s">
         <v>675</v>
       </c>
@@ -3598,7 +3883,7 @@
         <v>700</v>
       </c>
       <c r="T14" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="15" spans="1:22" x14ac:dyDescent="0.2">
@@ -3625,6 +3910,12 @@
         <f t="shared" si="0"/>
         <v>7.7</v>
       </c>
+      <c r="H15" s="4" t="s">
+        <v>815</v>
+      </c>
+      <c r="I15" t="s">
+        <v>24</v>
+      </c>
       <c r="K15" t="s">
         <v>675</v>
       </c>
@@ -3647,7 +3938,7 @@
         <v>700</v>
       </c>
       <c r="T15" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="16" spans="1:22" x14ac:dyDescent="0.2">
@@ -3674,6 +3965,12 @@
         <f t="shared" si="0"/>
         <v>30.5</v>
       </c>
+      <c r="H16" t="s">
+        <v>25</v>
+      </c>
+      <c r="I16" s="4" t="s">
+        <v>816</v>
+      </c>
       <c r="K16" t="s">
         <v>675</v>
       </c>
@@ -3696,7 +3993,7 @@
         <v>700</v>
       </c>
       <c r="T16" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="17" spans="1:20" x14ac:dyDescent="0.2">
@@ -3723,6 +4020,12 @@
         <f t="shared" si="0"/>
         <v>-7.9</v>
       </c>
+      <c r="H17" s="4" t="s">
+        <v>885</v>
+      </c>
+      <c r="I17" t="s">
+        <v>817</v>
+      </c>
       <c r="K17" t="s">
         <v>675</v>
       </c>
@@ -3745,7 +4048,7 @@
         <v>700</v>
       </c>
       <c r="T17" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="18" spans="1:20" x14ac:dyDescent="0.2">
@@ -3772,6 +4075,12 @@
         <f t="shared" si="0"/>
         <v>-22.6</v>
       </c>
+      <c r="H18" s="4" t="s">
+        <v>818</v>
+      </c>
+      <c r="I18" t="s">
+        <v>27</v>
+      </c>
       <c r="K18" t="s">
         <v>675</v>
       </c>
@@ -3794,7 +4103,7 @@
         <v>700</v>
       </c>
       <c r="T18" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="19" spans="1:20" x14ac:dyDescent="0.2">
@@ -4211,6 +4520,9 @@
       <c r="H26" s="6" t="s">
         <v>38</v>
       </c>
+      <c r="J26" s="4" t="s">
+        <v>819</v>
+      </c>
       <c r="K26" t="s">
         <v>667</v>
       </c>
@@ -4233,7 +4545,7 @@
         <v>699</v>
       </c>
       <c r="T26" t="s">
-        <v>703</v>
+        <v>728</v>
       </c>
     </row>
     <row r="27" spans="1:20" x14ac:dyDescent="0.2">
@@ -4539,6 +4851,9 @@
       <c r="H32" t="s">
         <v>43</v>
       </c>
+      <c r="I32" s="4" t="s">
+        <v>820</v>
+      </c>
       <c r="K32" t="s">
         <v>667</v>
       </c>
@@ -4561,7 +4876,7 @@
         <v>699</v>
       </c>
       <c r="T32" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="33" spans="1:20" x14ac:dyDescent="0.2">
@@ -4756,6 +5071,9 @@
       <c r="H36" s="4" t="s">
         <v>750</v>
       </c>
+      <c r="J36" s="4" t="s">
+        <v>821</v>
+      </c>
       <c r="K36" t="s">
         <v>667</v>
       </c>
@@ -4778,7 +5096,7 @@
         <v>699</v>
       </c>
       <c r="T36" t="s">
-        <v>703</v>
+        <v>728</v>
       </c>
     </row>
     <row r="37" spans="1:20" x14ac:dyDescent="0.2">
@@ -4863,6 +5181,9 @@
       <c r="H38" t="s">
         <v>49</v>
       </c>
+      <c r="I38" s="4" t="s">
+        <v>822</v>
+      </c>
       <c r="K38" t="s">
         <v>667</v>
       </c>
@@ -4885,7 +5206,7 @@
         <v>699</v>
       </c>
       <c r="T38" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="39" spans="1:20" x14ac:dyDescent="0.2">
@@ -6350,6 +6671,9 @@
       <c r="H65" t="s">
         <v>75</v>
       </c>
+      <c r="I65" s="4" t="s">
+        <v>823</v>
+      </c>
       <c r="K65" t="s">
         <v>667</v>
       </c>
@@ -6372,7 +6696,7 @@
         <v>699</v>
       </c>
       <c r="T65" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="66" spans="1:20" x14ac:dyDescent="0.2">
@@ -6896,6 +7220,12 @@
         <f t="shared" si="1"/>
         <v>64.3</v>
       </c>
+      <c r="H75" s="4" t="s">
+        <v>887</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>888</v>
+      </c>
       <c r="K75" t="s">
         <v>666</v>
       </c>
@@ -6918,7 +7248,7 @@
         <v>700</v>
       </c>
       <c r="T75" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="76" spans="1:20" x14ac:dyDescent="0.2">
@@ -6945,6 +7275,12 @@
         <f t="shared" si="1"/>
         <v>48.199999999999996</v>
       </c>
+      <c r="H76" t="s">
+        <v>86</v>
+      </c>
+      <c r="I76" s="4" t="s">
+        <v>889</v>
+      </c>
       <c r="K76" t="s">
         <v>666</v>
       </c>
@@ -6967,7 +7303,7 @@
         <v>700</v>
       </c>
       <c r="T76" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="77" spans="1:20" x14ac:dyDescent="0.2">
@@ -6994,6 +7330,12 @@
         <f t="shared" si="1"/>
         <v>-1.2999999999999989</v>
       </c>
+      <c r="H77" s="4" t="s">
+        <v>890</v>
+      </c>
+      <c r="I77" s="6" t="s">
+        <v>87</v>
+      </c>
       <c r="K77" t="s">
         <v>666</v>
       </c>
@@ -7016,7 +7358,7 @@
         <v>700</v>
       </c>
       <c r="T77" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="78" spans="1:20" x14ac:dyDescent="0.2">
@@ -7043,6 +7385,12 @@
         <f t="shared" si="1"/>
         <v>-9.9</v>
       </c>
+      <c r="H78" s="4" t="s">
+        <v>891</v>
+      </c>
+      <c r="I78" s="6" t="s">
+        <v>88</v>
+      </c>
       <c r="K78" t="s">
         <v>679</v>
       </c>
@@ -7065,7 +7413,7 @@
         <v>700</v>
       </c>
       <c r="T78" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="79" spans="1:20" x14ac:dyDescent="0.2">
@@ -7092,6 +7440,12 @@
         <f t="shared" si="1"/>
         <v>-0.69999999999999929</v>
       </c>
+      <c r="H79" s="4" t="s">
+        <v>892</v>
+      </c>
+      <c r="I79" s="6" t="s">
+        <v>89</v>
+      </c>
       <c r="K79" t="s">
         <v>666</v>
       </c>
@@ -7114,7 +7468,7 @@
         <v>700</v>
       </c>
       <c r="T79" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="80" spans="1:20" x14ac:dyDescent="0.2">
@@ -7141,6 +7495,12 @@
         <f t="shared" si="1"/>
         <v>28.200000000000003</v>
       </c>
+      <c r="H80" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="I80" s="4" t="s">
+        <v>893</v>
+      </c>
       <c r="K80" t="s">
         <v>666</v>
       </c>
@@ -7163,7 +7523,7 @@
         <v>700</v>
       </c>
       <c r="T80" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="81" spans="1:20" x14ac:dyDescent="0.2">
@@ -7190,6 +7550,12 @@
         <f t="shared" si="1"/>
         <v>23.4</v>
       </c>
+      <c r="H81" s="6" t="s">
+        <v>91</v>
+      </c>
+      <c r="I81" s="4" t="s">
+        <v>894</v>
+      </c>
       <c r="K81" t="s">
         <v>666</v>
       </c>
@@ -7212,7 +7578,7 @@
         <v>700</v>
       </c>
       <c r="T81" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="82" spans="1:20" x14ac:dyDescent="0.2">
@@ -7239,6 +7605,12 @@
         <f t="shared" si="1"/>
         <v>6.6000000000000005</v>
       </c>
+      <c r="H82" s="4" t="s">
+        <v>895</v>
+      </c>
+      <c r="I82" s="6" t="s">
+        <v>92</v>
+      </c>
       <c r="K82" t="s">
         <v>666</v>
       </c>
@@ -7261,7 +7633,7 @@
         <v>700</v>
       </c>
       <c r="T82" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="83" spans="1:20" x14ac:dyDescent="0.2">
@@ -8982,6 +9354,12 @@
         <f t="shared" si="1"/>
         <v>-7.2999999999999989</v>
       </c>
+      <c r="H117" s="4" t="s">
+        <v>824</v>
+      </c>
+      <c r="I117" s="4" t="s">
+        <v>825</v>
+      </c>
       <c r="K117" t="s">
         <v>677</v>
       </c>
@@ -9257,6 +9635,9 @@
       <c r="H122" t="s">
         <v>135</v>
       </c>
+      <c r="I122" s="4" t="s">
+        <v>826</v>
+      </c>
       <c r="K122" t="s">
         <v>677</v>
       </c>
@@ -9306,6 +9687,9 @@
         <f t="shared" si="1"/>
         <v>-12.700000000000001</v>
       </c>
+      <c r="H123" s="4" t="s">
+        <v>827</v>
+      </c>
       <c r="I123" s="6" t="s">
         <v>136</v>
       </c>
@@ -9471,6 +9855,9 @@
         <f t="shared" si="1"/>
         <v>-13.499999999999998</v>
       </c>
+      <c r="H126" s="4" t="s">
+        <v>828</v>
+      </c>
       <c r="I126" s="4" t="s">
         <v>142</v>
       </c>
@@ -9527,6 +9914,9 @@
       <c r="H127" s="4" t="s">
         <v>144</v>
       </c>
+      <c r="I127" s="4" t="s">
+        <v>829</v>
+      </c>
       <c r="K127" t="s">
         <v>677</v>
       </c>
@@ -9576,6 +9966,9 @@
         <f t="shared" si="1"/>
         <v>-5.6999999999999993</v>
       </c>
+      <c r="H128" s="4" t="s">
+        <v>830</v>
+      </c>
       <c r="I128" t="s">
         <v>145</v>
       </c>
@@ -12438,6 +12831,9 @@
         <f t="shared" si="2"/>
         <v>-1.0999999999999996</v>
       </c>
+      <c r="H182" s="4" t="s">
+        <v>831</v>
+      </c>
       <c r="I182" s="4" t="s">
         <v>798</v>
       </c>
@@ -12463,7 +12859,7 @@
         <v>809</v>
       </c>
       <c r="T182" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="183" spans="1:20" x14ac:dyDescent="0.2">
@@ -12490,6 +12886,12 @@
         <f t="shared" si="2"/>
         <v>-8.4</v>
       </c>
+      <c r="H183" s="4" t="s">
+        <v>865</v>
+      </c>
+      <c r="I183" t="s">
+        <v>243</v>
+      </c>
       <c r="K183" t="s">
         <v>676</v>
       </c>
@@ -12512,7 +12914,7 @@
         <v>700</v>
       </c>
       <c r="T183" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="184" spans="1:20" x14ac:dyDescent="0.2">
@@ -12539,6 +12941,12 @@
         <f t="shared" si="2"/>
         <v>26.700000000000003</v>
       </c>
+      <c r="H184" t="s">
+        <v>244</v>
+      </c>
+      <c r="I184" s="4" t="s">
+        <v>867</v>
+      </c>
       <c r="K184" t="s">
         <v>676</v>
       </c>
@@ -12561,7 +12969,7 @@
         <v>700</v>
       </c>
       <c r="T184" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="185" spans="1:20" x14ac:dyDescent="0.2">
@@ -12588,6 +12996,12 @@
         <f t="shared" si="2"/>
         <v>31.9</v>
       </c>
+      <c r="H185" t="s">
+        <v>245</v>
+      </c>
+      <c r="I185" s="4" t="s">
+        <v>868</v>
+      </c>
       <c r="K185" t="s">
         <v>676</v>
       </c>
@@ -12610,7 +13024,7 @@
         <v>700</v>
       </c>
       <c r="T185" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="186" spans="1:20" x14ac:dyDescent="0.2">
@@ -12637,6 +13051,12 @@
         <f t="shared" si="2"/>
         <v>81.600000000000009</v>
       </c>
+      <c r="H186" t="s">
+        <v>246</v>
+      </c>
+      <c r="I186" s="4" t="s">
+        <v>869</v>
+      </c>
       <c r="K186" t="s">
         <v>676</v>
       </c>
@@ -12659,7 +13079,7 @@
         <v>700</v>
       </c>
       <c r="T186" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="187" spans="1:20" x14ac:dyDescent="0.2">
@@ -12686,6 +13106,12 @@
         <f t="shared" si="2"/>
         <v>41.5</v>
       </c>
+      <c r="H187" t="s">
+        <v>866</v>
+      </c>
+      <c r="I187" s="4" t="s">
+        <v>870</v>
+      </c>
       <c r="K187" t="s">
         <v>676</v>
       </c>
@@ -12708,7 +13134,7 @@
         <v>700</v>
       </c>
       <c r="T187" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="188" spans="1:20" x14ac:dyDescent="0.2">
@@ -12735,6 +13161,12 @@
         <f t="shared" si="2"/>
         <v>14.100000000000001</v>
       </c>
+      <c r="H188" t="s">
+        <v>248</v>
+      </c>
+      <c r="I188" s="4" t="s">
+        <v>871</v>
+      </c>
       <c r="K188" t="s">
         <v>676</v>
       </c>
@@ -12757,7 +13189,7 @@
         <v>700</v>
       </c>
       <c r="T188" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="189" spans="1:20" x14ac:dyDescent="0.2">
@@ -12784,6 +13216,12 @@
         <f t="shared" si="2"/>
         <v>67</v>
       </c>
+      <c r="H189" t="s">
+        <v>249</v>
+      </c>
+      <c r="I189" s="4" t="s">
+        <v>872</v>
+      </c>
       <c r="K189" t="s">
         <v>676</v>
       </c>
@@ -12806,7 +13244,7 @@
         <v>700</v>
       </c>
       <c r="T189" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="190" spans="1:20" x14ac:dyDescent="0.2">
@@ -12833,6 +13271,12 @@
         <f t="shared" si="2"/>
         <v>64.199999999999989</v>
       </c>
+      <c r="H190" t="s">
+        <v>250</v>
+      </c>
+      <c r="I190" s="4" t="s">
+        <v>873</v>
+      </c>
       <c r="K190" t="s">
         <v>676</v>
       </c>
@@ -12855,7 +13299,7 @@
         <v>700</v>
       </c>
       <c r="T190" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="191" spans="1:20" x14ac:dyDescent="0.2">
@@ -16005,6 +16449,9 @@
       <c r="H252" t="s">
         <v>319</v>
       </c>
+      <c r="I252" s="4" t="s">
+        <v>832</v>
+      </c>
       <c r="K252" t="s">
         <v>676</v>
       </c>
@@ -16027,7 +16474,7 @@
         <v>700</v>
       </c>
       <c r="T252" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="253" spans="1:20" x14ac:dyDescent="0.2">
@@ -16387,6 +16834,12 @@
         <f t="shared" si="4"/>
         <v>-1.6999999999999993</v>
       </c>
+      <c r="H259" s="4" t="s">
+        <v>833</v>
+      </c>
+      <c r="I259" s="6" t="s">
+        <v>326</v>
+      </c>
       <c r="K259" t="s">
         <v>676</v>
       </c>
@@ -16436,6 +16889,12 @@
         <f t="shared" si="4"/>
         <v>-5.5</v>
       </c>
+      <c r="H260" s="4" t="s">
+        <v>834</v>
+      </c>
+      <c r="I260" s="6" t="s">
+        <v>327</v>
+      </c>
       <c r="K260" t="s">
         <v>676</v>
       </c>
@@ -16485,6 +16944,12 @@
         <f t="shared" si="4"/>
         <v>4.1000000000000005</v>
       </c>
+      <c r="H261" t="s">
+        <v>328</v>
+      </c>
+      <c r="I261" s="4" t="s">
+        <v>835</v>
+      </c>
       <c r="K261" t="s">
         <v>676</v>
       </c>
@@ -16534,6 +16999,12 @@
         <f t="shared" si="4"/>
         <v>9.7000000000000011</v>
       </c>
+      <c r="H262" t="s">
+        <v>329</v>
+      </c>
+      <c r="I262" s="4" t="s">
+        <v>836</v>
+      </c>
       <c r="K262" t="s">
         <v>676</v>
       </c>
@@ -16583,6 +17054,12 @@
         <f t="shared" si="4"/>
         <v>50.6</v>
       </c>
+      <c r="H263" t="s">
+        <v>330</v>
+      </c>
+      <c r="I263" s="4" t="s">
+        <v>837</v>
+      </c>
       <c r="K263" t="s">
         <v>676</v>
       </c>
@@ -16632,6 +17109,12 @@
         <f t="shared" si="4"/>
         <v>14.8</v>
       </c>
+      <c r="H264" t="s">
+        <v>331</v>
+      </c>
+      <c r="I264" s="4" t="s">
+        <v>838</v>
+      </c>
       <c r="K264" t="s">
         <v>676</v>
       </c>
@@ -16681,6 +17164,12 @@
         <f t="shared" si="4"/>
         <v>54.3</v>
       </c>
+      <c r="H265" s="4" t="s">
+        <v>839</v>
+      </c>
+      <c r="I265" s="4" t="s">
+        <v>840</v>
+      </c>
       <c r="K265" t="s">
         <v>676</v>
       </c>
@@ -16730,6 +17219,12 @@
         <f t="shared" si="4"/>
         <v>52.4</v>
       </c>
+      <c r="H266" t="s">
+        <v>333</v>
+      </c>
+      <c r="I266" s="4" t="s">
+        <v>841</v>
+      </c>
       <c r="K266" t="s">
         <v>676</v>
       </c>
@@ -16779,6 +17274,12 @@
         <f t="shared" si="4"/>
         <v>49</v>
       </c>
+      <c r="H267" t="s">
+        <v>334</v>
+      </c>
+      <c r="I267" s="4" t="s">
+        <v>842</v>
+      </c>
       <c r="K267" t="s">
         <v>676</v>
       </c>
@@ -16828,6 +17329,12 @@
         <f t="shared" si="4"/>
         <v>68.8</v>
       </c>
+      <c r="H268" s="4" t="s">
+        <v>843</v>
+      </c>
+      <c r="I268" s="4" t="s">
+        <v>844</v>
+      </c>
       <c r="K268" t="s">
         <v>676</v>
       </c>
@@ -16877,6 +17384,12 @@
         <f t="shared" si="4"/>
         <v>-16</v>
       </c>
+      <c r="H269" s="4" t="s">
+        <v>845</v>
+      </c>
+      <c r="I269" s="6" t="s">
+        <v>336</v>
+      </c>
       <c r="K269" t="s">
         <v>676</v>
       </c>
@@ -16926,6 +17439,12 @@
         <f t="shared" si="4"/>
         <v>72</v>
       </c>
+      <c r="H270" s="4" t="s">
+        <v>846</v>
+      </c>
+      <c r="I270" s="4" t="s">
+        <v>847</v>
+      </c>
       <c r="K270" t="s">
         <v>676</v>
       </c>
@@ -16975,6 +17494,12 @@
         <f t="shared" si="4"/>
         <v>67.7</v>
       </c>
+      <c r="H271" s="4" t="s">
+        <v>848</v>
+      </c>
+      <c r="I271" s="4" t="s">
+        <v>849</v>
+      </c>
       <c r="K271" t="s">
         <v>676</v>
       </c>
@@ -17024,6 +17549,12 @@
         <f t="shared" si="4"/>
         <v>40.200000000000003</v>
       </c>
+      <c r="H272" s="6" t="s">
+        <v>339</v>
+      </c>
+      <c r="I272" s="4" t="s">
+        <v>850</v>
+      </c>
       <c r="K272" t="s">
         <v>676</v>
       </c>
@@ -17073,6 +17604,12 @@
         <f t="shared" si="4"/>
         <v>56.699999999999996</v>
       </c>
+      <c r="H273" s="6" t="s">
+        <v>340</v>
+      </c>
+      <c r="I273" s="4" t="s">
+        <v>851</v>
+      </c>
       <c r="K273" t="s">
         <v>676</v>
       </c>
@@ -17122,6 +17659,12 @@
         <f t="shared" si="4"/>
         <v>41.5</v>
       </c>
+      <c r="H274" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="I274" s="4" t="s">
+        <v>852</v>
+      </c>
       <c r="K274" t="s">
         <v>663</v>
       </c>
@@ -17171,6 +17714,12 @@
         <f t="shared" si="4"/>
         <v>9</v>
       </c>
+      <c r="H275" s="4" t="s">
+        <v>853</v>
+      </c>
+      <c r="I275" s="6" t="s">
+        <v>342</v>
+      </c>
       <c r="K275" t="s">
         <v>663</v>
       </c>
@@ -17220,6 +17769,12 @@
         <f t="shared" si="4"/>
         <v>11.7</v>
       </c>
+      <c r="H276" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="I276" s="4" t="s">
+        <v>854</v>
+      </c>
       <c r="K276" t="s">
         <v>663</v>
       </c>
@@ -17269,6 +17824,12 @@
         <f t="shared" si="4"/>
         <v>10.200000000000001</v>
       </c>
+      <c r="H277" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="I277" s="4" t="s">
+        <v>855</v>
+      </c>
       <c r="K277" t="s">
         <v>663</v>
       </c>
@@ -17319,6 +17880,12 @@
         <f t="shared" si="4"/>
         <v>22.6</v>
       </c>
+      <c r="H278" s="6" t="s">
+        <v>345</v>
+      </c>
+      <c r="I278" s="4" t="s">
+        <v>856</v>
+      </c>
       <c r="K278" t="s">
         <v>663</v>
       </c>
@@ -17368,6 +17935,12 @@
         <f t="shared" si="4"/>
         <v>-12.299999999999999</v>
       </c>
+      <c r="H279" s="4" t="s">
+        <v>857</v>
+      </c>
+      <c r="I279" s="4" t="s">
+        <v>858</v>
+      </c>
       <c r="K279" t="s">
         <v>663</v>
       </c>
@@ -17417,6 +17990,12 @@
         <f t="shared" si="4"/>
         <v>16.100000000000001</v>
       </c>
+      <c r="H280" s="6" t="s">
+        <v>347</v>
+      </c>
+      <c r="I280" s="4" t="s">
+        <v>859</v>
+      </c>
       <c r="K280" t="s">
         <v>663</v>
       </c>
@@ -17466,6 +18045,12 @@
         <f t="shared" si="4"/>
         <v>-12.6</v>
       </c>
+      <c r="H281" s="4" t="s">
+        <v>860</v>
+      </c>
+      <c r="I281" s="6" t="s">
+        <v>348</v>
+      </c>
       <c r="K281" t="s">
         <v>663</v>
       </c>
@@ -17515,6 +18100,12 @@
         <f t="shared" si="4"/>
         <v>-14.700000000000003</v>
       </c>
+      <c r="H282" s="4" t="s">
+        <v>861</v>
+      </c>
+      <c r="I282" s="6" t="s">
+        <v>349</v>
+      </c>
       <c r="K282" t="s">
         <v>663</v>
       </c>
@@ -17564,6 +18155,12 @@
         <f t="shared" si="4"/>
         <v>26.799999999999997</v>
       </c>
+      <c r="H283" s="6" t="s">
+        <v>862</v>
+      </c>
+      <c r="I283" s="4" t="s">
+        <v>863</v>
+      </c>
       <c r="K283" t="s">
         <v>663</v>
       </c>
@@ -17613,6 +18210,12 @@
         <f t="shared" si="4"/>
         <v>27.700000000000003</v>
       </c>
+      <c r="H284" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="I284" s="4" t="s">
+        <v>864</v>
+      </c>
       <c r="K284" t="s">
         <v>663</v>
       </c>
@@ -18436,6 +19039,9 @@
         <f t="shared" si="4"/>
         <v>-28.4</v>
       </c>
+      <c r="H299" s="4" t="s">
+        <v>897</v>
+      </c>
       <c r="I299" t="s">
         <v>793</v>
       </c>
@@ -18461,7 +19067,7 @@
         <v>700</v>
       </c>
       <c r="T299" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="300" spans="1:20" x14ac:dyDescent="0.2">
@@ -20952,7 +21558,12 @@
         <f t="shared" si="5"/>
         <v>-4.6999999999999993</v>
       </c>
-      <c r="H345" s="4"/>
+      <c r="H345" s="4" t="s">
+        <v>874</v>
+      </c>
+      <c r="I345" t="s">
+        <v>875</v>
+      </c>
       <c r="K345" t="s">
         <v>677</v>
       </c>
@@ -20975,7 +21586,7 @@
         <v>700</v>
       </c>
       <c r="T345" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="346" spans="1:20" x14ac:dyDescent="0.2">
@@ -21002,6 +21613,9 @@
         <f t="shared" si="5"/>
         <v>-5.6</v>
       </c>
+      <c r="H346" s="4" t="s">
+        <v>876</v>
+      </c>
       <c r="I346" t="s">
         <v>467</v>
       </c>
@@ -21027,7 +21641,7 @@
         <v>700</v>
       </c>
       <c r="T346" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="347" spans="1:20" x14ac:dyDescent="0.2">
@@ -21054,7 +21668,7 @@
         <f t="shared" si="5"/>
         <v>-34.6</v>
       </c>
-      <c r="H347" t="s">
+      <c r="H347" s="4" t="s">
         <v>800</v>
       </c>
       <c r="I347" t="s">
@@ -23947,6 +24561,12 @@
         <f t="shared" si="6"/>
         <v>32</v>
       </c>
+      <c r="H400" s="4" t="s">
+        <v>877</v>
+      </c>
+      <c r="I400" s="4" t="s">
+        <v>878</v>
+      </c>
       <c r="K400" t="s">
         <v>666</v>
       </c>
@@ -23969,7 +24589,7 @@
         <v>700</v>
       </c>
       <c r="T400" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="401" spans="1:20" x14ac:dyDescent="0.2">
@@ -23996,6 +24616,12 @@
         <f t="shared" si="6"/>
         <v>-20.5</v>
       </c>
+      <c r="H401" s="4" t="s">
+        <v>879</v>
+      </c>
+      <c r="I401" s="6" t="s">
+        <v>570</v>
+      </c>
       <c r="K401" t="s">
         <v>666</v>
       </c>
@@ -24018,7 +24644,7 @@
         <v>700</v>
       </c>
       <c r="T401" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="402" spans="1:20" x14ac:dyDescent="0.2">
@@ -24045,6 +24671,12 @@
         <f t="shared" si="6"/>
         <v>-32.9</v>
       </c>
+      <c r="H402" s="4" t="s">
+        <v>880</v>
+      </c>
+      <c r="I402" s="6" t="s">
+        <v>571</v>
+      </c>
       <c r="K402" t="s">
         <v>666</v>
       </c>
@@ -24067,7 +24699,7 @@
         <v>700</v>
       </c>
       <c r="T402" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="403" spans="1:20" x14ac:dyDescent="0.2">
@@ -24094,6 +24726,12 @@
         <f t="shared" si="6"/>
         <v>-24</v>
       </c>
+      <c r="H403" s="4" t="s">
+        <v>881</v>
+      </c>
+      <c r="I403" s="6" t="s">
+        <v>572</v>
+      </c>
       <c r="K403" t="s">
         <v>666</v>
       </c>
@@ -24116,7 +24754,7 @@
         <v>700</v>
       </c>
       <c r="T403" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
     </row>
     <row r="404" spans="1:20" x14ac:dyDescent="0.2">

</xml_diff>